<commit_message>
Update index to 24159; add Excel report with 16 businesses (rows 24128-24159)
Processed addresses:
- שמואל הנגיד 14, 15, 17, 19, 20, 25, 9
- שמורק 1, 7, 10, 12, 14, 16, 18
- שמחת כהן 5-23 (batch)

16 verified businesses added to today's Excel report.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pBRKs8HcAHNyvncjCSQGM
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:13-09-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:13-09-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="נכסים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,24 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,46 +427,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>כתובת</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>שכונה</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>סוג עסק</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>דירוג אינדיקציה</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>קישור 1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>קישור 2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>קישור 3</t>
         </is>
@@ -721,6 +745,266 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>צבעי שלום</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>שמואל הנביא 5, ירושלים</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>חנות צבעים</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/25991761</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>גת רחמים</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>שמואל הנביא 68, ירושלים</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>אמני בידור</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/74890080/3310</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/25854253</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>מרכז אמבר ללימוד אנגלית</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>שמואל הנגיד 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>לימודי שפות</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80051587/8570</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/24353995</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ד"ר חנן רפפורט</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>שמואל הנגיד 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>פסיכולוגים קליניים</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/1984240/40270</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TPS Israel's News Agency</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>שמואל הנגיד 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>סוכנות חדשות</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/27422068</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ד"ר קלאפהולץ לורנט</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>שמואל הנגיד 19, ירושלים</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>רפואה</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/6940348</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>יד שרה</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>שמואל הנגיד 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ארגון סיוע</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/26964385</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>תריסי ניר גואטה</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>שמורק 10, ירושלים</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>קרית היובל</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>תריסים</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/25991386</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/71676460/52080</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>